<commit_message>
chore(ro-crate): sync from Google Sheets
</commit_message>
<xml_diff>
--- a/ro-crate/ro-crate-metadata.xlsx
+++ b/ro-crate/ro-crate-metadata.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="702" uniqueCount="328">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="729" uniqueCount="338">
   <si>
     <t>Name</t>
   </si>
@@ -92,7 +92,7 @@
     <t>pcdm:hasMember</t>
   </si>
   <si>
-    <t>["arcp://name,AnonymisingELANFiles", "arcp://name,CollocationAnalyser", "arcp://name,CollocationCalculator", "arcp://name,ConcordanceExplorer", "arcp://name,Concordancer", "arcp://name,Crate-O", "arcp://name,Discursis", "arcp://name,DocumentSimilarity", "arcp://name,ELANAnnotationSplitter", "arcp://name,ELANAudioSegmentation", "arcp://name,ELANCommander", "arcp://name,ELANInventory", "arcp://name,ELANReplacer", "arcp://name,FileRenamer", "arcp://name,ImageDatasetExplorer", "arcp://name,KeywordFinder", "arcp://name,KeywordExtractor", "arcp://name,KeywordsAnalysis", "arcp://name,Lameta", "arcp://name,NetworkVisualiser", "arcp://name,Part-of-SpeechTagger", "arcp://name,POSTagger", "arcp://name,QuotationTool", "arcp://name,SemanticTaggerEnglish", "arcp://name,SentimentExplorer", "arcp://name,SentimentExplorerbrowser-based", "arcp://name,TextCleaner", "arcp://name,TextCleanerbrowser-based", "arcp://name,TopicExplorer", "arcp://name,TopicDetector", "arcp://name,WordFinder", "arcp://name,WordWebber", "https://data.ldaca.edu.au/object?_id=https://github.com/Australian-Text-Analytics-Platform/cooee/blob/main/cooee.ipynb", "https://github.com/Australian-Text-Analytics-Platform/farms-to-freeways", "https://data.ldaca.edu.au/object?_id=https%3A%2F%2Fgithub.com%2FAustralian-Text-Analytics-Platform%2Fnotebook-ausreddit%2Fblob%2Fmain%2Fexploration.ipynb", "https://data.ldaca.edu.au/object?_id=https%3A%2F%2Fgithub.com%2FAustralian-Text-Analytics-Platform%2Fnotebook-twittersphere%2Fblob%2Fmain%2Fexploration.ipynb"]</t>
+    <t>["arcp://name,AnonymisingELANFiles", "arcp://name,CollocationAnalyser", "arcp://name,CollocationCalculator", "arcp://name,ConcordanceExplorer", "arcp://name,Concordancer", "arcp://name,Crate-O", "arcp://name,Discursis", "arcp://name,DocumentSimilarity", "arcp://name,ELANAnnotationSplitter", "arcp://name,ELANAudioSegmentation", "arcp://name,ELANCommander", "arcp://name,ELANInventory", "arcp://name,ELANReplacer", "arcp://name,FileRenamer", "arcp://name,ImageDatasetExplorer", "arcp://name,KeywordFinder", "arcp://name,KeywordExtractor", "arcp://name,KeywordsAnalysis", "arcp://name,Lameta", "arcp://name,NetworkVisualiser", "arcp://name,Part-of-SpeechTagger", "arcp://name,POSTagger", "arcp://name,QuotationTool", "arcp://name,SemanticTaggerEnglish", "arcp://name,SentimentExplorer", "arcp://name,SentimentExplorerbrowser-based", "arcp://name,TextCleaner", "arcp://name,TextCleanerbrowser-based", "arcp://name,TopicExplorer", "arcp://name,TopicDetector", "arcp://name,WordFinder", "arcp://name,WordWebber", "arcp://name,TopSBM", "arcp://name,SemanticTaggermultilingual", "https://data.ldaca.edu.au/object?_id=https://github.com/Australian-Text-Analytics-Platform/cooee/blob/main/cooee.ipynb", "https://github.com/Australian-Text-Analytics-Platform/farms-to-freeways", "https://data.ldaca.edu.au/object?_id=https%3A%2F%2Fgithub.com%2FAustralian-Text-Analytics-Platform%2Fnotebook-ausreddit%2Fblob%2Fmain%2Fexploration.ipynb", "https://data.ldaca.edu.au/object?_id=https%3A%2F%2Fgithub.com%2FAustralian-Text-Analytics-Platform%2Fnotebook-twittersphere%2Fblob%2Fmain%2Fexploration.ipynb"]</t>
   </si>
   <si>
     <t>hasPart</t>
@@ -536,7 +536,7 @@
     <t>https://raw.githubusercontent.com/Australian-Text-Analytics-Platform/discursis/master/docs/Discursis%20User%20Guide.pdf</t>
   </si>
   <si>
-    <t>Not provided</t>
+    <t>object Object</t>
   </si>
   <si>
     <t>Based on Angus et al</t>
@@ -735,9 +735,6 @@
     <t>https://www.elararchive.org/uncategorized/SO_7557c4dd-1c83-485c-b95c-c0a292cfc42c/</t>
   </si>
   <si>
-    <t>object Object</t>
-  </si>
-  <si>
     <t>arcp://name,NetworkVisualiser</t>
   </si>
   <si>
@@ -813,6 +810,9 @@
     <t>https://github.com/Australian-Text-Analytics-Platform/semantic-tagger/blob/main/documents/semtag_help_pages.pdf</t>
   </si>
   <si>
+    <t>Jufri, Sony &amp; Sun, Chao (2022). Semantic Tagger. v1.0. Australian Text Analytics Platform. Software. https://github.com/Australian-Text-Analytics-Platform/semantic-tagger</t>
+  </si>
+  <si>
     <t>arcp://name,SentimentExplorer</t>
   </si>
   <si>
@@ -898,6 +898,36 @@
   </si>
   <si>
     <t>"images/word-webber.png"</t>
+  </si>
+  <si>
+    <t>arcp://name,TopSBM</t>
+  </si>
+  <si>
+    <t>TopSBM</t>
+  </si>
+  <si>
+    <t>"https://orcid.org/0000-0002-1428-2649"</t>
+  </si>
+  <si>
+    <t>https://github.com/Australian-Text-Analytics-Platform/topsbm</t>
+  </si>
+  <si>
+    <t>Topic modelling approach that infers a hierarchy of topic clusters and word clusters in your Corpus in a non-parametric manner by leveraging stochastic block models.</t>
+  </si>
+  <si>
+    <t>arcp://name,SemanticTaggermultilingual</t>
+  </si>
+  <si>
+    <t>Semantic Tagger (multilingual)</t>
+  </si>
+  <si>
+    <t>https://github.com/Australian-Text-Analytics-Platform/semantic-tagger/tree/multi-lingual</t>
+  </si>
+  <si>
+    <t>With the multilingual Semantic Tagger, you can use Python Multilingual Ucrel Semantic Analysis System (PyMUSAS) to tag your text so you can extract token level semantic tags from the tagged text. Supports Chinese, Italian and Spanish languages.</t>
+  </si>
+  <si>
+    <t>https://github.com/Australian-Text-Analytics-Platform/semantic-tagger/blob/multi-lingual/documents/semtag_help_pages.pdf</t>
   </si>
   <si>
     <t>https://data.ldaca.edu.au/object?_id=https://github.com/Australian-Text-Analytics-Platform/cooee/blob/main/cooee.ipynb</t>
@@ -2136,7 +2166,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:S37"/>
+  <dimension ref="A1:S39"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="19" width="20" customWidth="1"/>
@@ -3016,12 +3046,12 @@
         <v>237</v>
       </c>
       <c r="P20" t="s">
-        <v>238</v>
+        <v>172</v>
       </c>
     </row>
     <row r="21" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B21" t="s">
         <v>120</v>
@@ -3033,7 +3063,7 @@
         <v>34</v>
       </c>
       <c r="E21" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="F21" t="s">
         <v>13</v>
@@ -3051,18 +3081,18 @@
         <v>134</v>
       </c>
       <c r="K21" t="s">
+        <v>240</v>
+      </c>
+      <c r="L21" t="s">
         <v>241</v>
       </c>
-      <c r="L21" t="s">
+      <c r="Q21" t="s">
         <v>242</v>
-      </c>
-      <c r="Q21" t="s">
-        <v>243</v>
       </c>
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B22" t="s">
         <v>120</v>
@@ -3074,7 +3104,7 @@
         <v>34</v>
       </c>
       <c r="E22" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="F22" t="s">
         <v>13</v>
@@ -3092,7 +3122,7 @@
         <v>134</v>
       </c>
       <c r="K22" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="L22" t="s">
         <v>136</v>
@@ -3100,7 +3130,7 @@
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B23" t="s">
         <v>120</v>
@@ -3112,7 +3142,7 @@
         <v>34</v>
       </c>
       <c r="E23" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="F23" t="s">
         <v>13</v>
@@ -3130,18 +3160,18 @@
         <v>140</v>
       </c>
       <c r="K23" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="L23" t="s">
         <v>136</v>
       </c>
       <c r="N23" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="24" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="B24" t="s">
         <v>120</v>
@@ -3153,7 +3183,7 @@
         <v>34</v>
       </c>
       <c r="E24" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="F24" t="s">
         <v>13</v>
@@ -3168,30 +3198,30 @@
         <v>125</v>
       </c>
       <c r="J24" t="s">
+        <v>252</v>
+      </c>
+      <c r="K24" t="s">
         <v>253</v>
-      </c>
-      <c r="K24" t="s">
-        <v>254</v>
       </c>
       <c r="L24" t="s">
         <v>152</v>
       </c>
       <c r="M24" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="N24" t="s">
+        <v>254</v>
+      </c>
+      <c r="O24" t="s">
         <v>255</v>
       </c>
-      <c r="O24" t="s">
+      <c r="P24" t="s">
         <v>256</v>
-      </c>
-      <c r="P24" t="s">
-        <v>257</v>
       </c>
     </row>
     <row r="25" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B25" t="s">
         <v>120</v>
@@ -3203,7 +3233,7 @@
         <v>34</v>
       </c>
       <c r="E25" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="F25" t="s">
         <v>13</v>
@@ -3218,25 +3248,25 @@
         <v>125</v>
       </c>
       <c r="J25" t="s">
+        <v>259</v>
+      </c>
+      <c r="K25" t="s">
         <v>260</v>
-      </c>
-      <c r="K25" t="s">
-        <v>261</v>
       </c>
       <c r="L25" t="s">
         <v>152</v>
       </c>
       <c r="M25" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="N25" t="s">
+        <v>261</v>
+      </c>
+      <c r="O25" t="s">
         <v>262</v>
       </c>
-      <c r="O25" t="s">
+      <c r="P25" t="s">
         <v>263</v>
-      </c>
-      <c r="P25" t="s">
-        <v>238</v>
       </c>
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.25">
@@ -3552,16 +3582,16 @@
         <v>291</v>
       </c>
       <c r="L33" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="N33" t="s">
         <v>292</v>
       </c>
       <c r="Q33" t="s">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="34" spans="1:19" x14ac:dyDescent="0.25">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="34" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>293</v>
       </c>
@@ -3569,175 +3599,260 @@
         <v>120</v>
       </c>
       <c r="C34" t="s">
+        <v>121</v>
+      </c>
+      <c r="D34" t="s">
+        <v>34</v>
+      </c>
+      <c r="E34" t="s">
         <v>294</v>
-      </c>
-      <c r="D34" t="s">
-        <v>34</v>
-      </c>
-      <c r="E34" t="s">
-        <v>295</v>
       </c>
       <c r="F34" t="s">
         <v>13</v>
       </c>
       <c r="G34" t="s">
-        <v>123</v>
+        <v>148</v>
       </c>
       <c r="H34" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="I34" t="s">
         <v>125</v>
       </c>
       <c r="J34" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="K34" t="s">
         <v>297</v>
       </c>
-      <c r="M34" t="s">
+      <c r="L34" t="s">
+        <v>152</v>
+      </c>
+      <c r="P34" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="35" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
         <v>298</v>
-      </c>
-      <c r="R34" t="s">
-        <v>299</v>
-      </c>
-      <c r="S34" t="s">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="35" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>301</v>
       </c>
       <c r="B35" t="s">
         <v>120</v>
       </c>
       <c r="C35" t="s">
-        <v>294</v>
+        <v>121</v>
       </c>
       <c r="D35" t="s">
         <v>34</v>
       </c>
       <c r="E35" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="F35" t="s">
-        <v>303</v>
+        <v>13</v>
       </c>
       <c r="G35" t="s">
-        <v>123</v>
+        <v>148</v>
       </c>
       <c r="H35" t="s">
-        <v>304</v>
+        <v>176</v>
       </c>
       <c r="I35" t="s">
         <v>125</v>
       </c>
       <c r="J35" t="s">
+        <v>300</v>
+      </c>
+      <c r="K35" t="s">
         <v>301</v>
       </c>
       <c r="L35" t="s">
-        <v>305</v>
-      </c>
-      <c r="M35" t="s">
-        <v>301</v>
-      </c>
-      <c r="R35" t="s">
-        <v>306</v>
-      </c>
-      <c r="S35" t="s">
-        <v>300</v>
+        <v>152</v>
+      </c>
+      <c r="O35" t="s">
+        <v>302</v>
+      </c>
+      <c r="P35" t="s">
+        <v>172</v>
       </c>
     </row>
     <row r="36" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>307</v>
+        <v>303</v>
       </c>
       <c r="B36" t="s">
         <v>120</v>
       </c>
       <c r="C36" t="s">
-        <v>294</v>
+        <v>304</v>
       </c>
       <c r="D36" t="s">
         <v>34</v>
       </c>
       <c r="E36" t="s">
-        <v>308</v>
+        <v>305</v>
+      </c>
+      <c r="F36" t="s">
+        <v>13</v>
       </c>
       <c r="G36" t="s">
-        <v>309</v>
+        <v>123</v>
       </c>
       <c r="H36" t="s">
-        <v>310</v>
+        <v>306</v>
       </c>
       <c r="I36" t="s">
         <v>125</v>
       </c>
       <c r="J36" t="s">
+        <v>303</v>
+      </c>
+      <c r="K36" t="s">
         <v>307</v>
       </c>
-      <c r="K36" t="s">
-        <v>311</v>
-      </c>
-      <c r="L36" t="s">
-        <v>312</v>
-      </c>
       <c r="M36" t="s">
-        <v>313</v>
+        <v>308</v>
       </c>
       <c r="R36" t="s">
-        <v>314</v>
+        <v>309</v>
       </c>
       <c r="S36" t="s">
-        <v>300</v>
+        <v>310</v>
       </c>
     </row>
     <row r="37" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>315</v>
+        <v>311</v>
       </c>
       <c r="B37" t="s">
         <v>120</v>
       </c>
       <c r="C37" t="s">
-        <v>294</v>
+        <v>304</v>
       </c>
       <c r="D37" t="s">
         <v>34</v>
       </c>
       <c r="E37" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="F37" t="s">
-        <v>13</v>
+        <v>313</v>
       </c>
       <c r="G37" t="s">
-        <v>309</v>
+        <v>123</v>
       </c>
       <c r="H37" t="s">
-        <v>310</v>
+        <v>314</v>
       </c>
       <c r="I37" t="s">
         <v>125</v>
       </c>
       <c r="J37" t="s">
+        <v>311</v>
+      </c>
+      <c r="L37" t="s">
         <v>315</v>
       </c>
-      <c r="K37" t="s">
+      <c r="M37" t="s">
+        <v>311</v>
+      </c>
+      <c r="R37" t="s">
+        <v>316</v>
+      </c>
+      <c r="S37" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="38" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
         <v>317</v>
       </c>
-      <c r="L37" t="s">
-        <v>312</v>
-      </c>
-      <c r="M37" t="s">
+      <c r="B38" t="s">
+        <v>120</v>
+      </c>
+      <c r="C38" t="s">
+        <v>304</v>
+      </c>
+      <c r="D38" t="s">
+        <v>34</v>
+      </c>
+      <c r="E38" t="s">
         <v>318</v>
       </c>
-      <c r="R37" t="s">
+      <c r="G38" t="s">
         <v>319</v>
       </c>
-      <c r="S37" t="s">
-        <v>300</v>
+      <c r="H38" t="s">
+        <v>320</v>
+      </c>
+      <c r="I38" t="s">
+        <v>125</v>
+      </c>
+      <c r="J38" t="s">
+        <v>317</v>
+      </c>
+      <c r="K38" t="s">
+        <v>321</v>
+      </c>
+      <c r="L38" t="s">
+        <v>322</v>
+      </c>
+      <c r="M38" t="s">
+        <v>323</v>
+      </c>
+      <c r="R38" t="s">
+        <v>324</v>
+      </c>
+      <c r="S38" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="39" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>325</v>
+      </c>
+      <c r="B39" t="s">
+        <v>120</v>
+      </c>
+      <c r="C39" t="s">
+        <v>304</v>
+      </c>
+      <c r="D39" t="s">
+        <v>34</v>
+      </c>
+      <c r="E39" t="s">
+        <v>326</v>
+      </c>
+      <c r="F39" t="s">
+        <v>13</v>
+      </c>
+      <c r="G39" t="s">
+        <v>319</v>
+      </c>
+      <c r="H39" t="s">
+        <v>320</v>
+      </c>
+      <c r="I39" t="s">
+        <v>125</v>
+      </c>
+      <c r="J39" t="s">
+        <v>325</v>
+      </c>
+      <c r="K39" t="s">
+        <v>327</v>
+      </c>
+      <c r="L39" t="s">
+        <v>322</v>
+      </c>
+      <c r="M39" t="s">
+        <v>328</v>
+      </c>
+      <c r="R39" t="s">
+        <v>329</v>
+      </c>
+      <c r="S39" t="s">
+        <v>310</v>
       </c>
     </row>
   </sheetData>
@@ -3767,46 +3882,46 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>320</v>
+        <v>330</v>
       </c>
       <c r="B2" t="s">
-        <v>321</v>
+        <v>331</v>
       </c>
       <c r="C2" t="s">
-        <v>322</v>
+        <v>332</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>323</v>
+        <v>333</v>
       </c>
       <c r="B3" t="s">
-        <v>324</v>
+        <v>334</v>
       </c>
       <c r="C3" t="s">
-        <v>322</v>
+        <v>332</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>325</v>
+        <v>335</v>
       </c>
       <c r="B4" t="s">
-        <v>238</v>
+        <v>172</v>
       </c>
       <c r="C4" t="s">
-        <v>322</v>
+        <v>332</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>326</v>
+        <v>336</v>
       </c>
       <c r="B5" t="s">
-        <v>327</v>
+        <v>337</v>
       </c>
       <c r="C5" t="s">
-        <v>322</v>
+        <v>332</v>
       </c>
     </row>
   </sheetData>

</xml_diff>